<commit_message>
[ Data ] Update player default attack speed
</commit_message>
<xml_diff>
--- a/Assets/RawData/Excel/Player/PlayerStatData.xlsx
+++ b/Assets/RawData/Excel/Player/PlayerStatData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\TinyHero\Assets\RawData\Excel\Player\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F98E60-6545-4969-BD39-19133F77E8D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E047CC7-4A3A-46A0-AA62-7A9139ACE9A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -486,7 +486,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <v>4.5</v>

</xml_diff>